<commit_message>
coordinates moved to excel
</commit_message>
<xml_diff>
--- a/Historical_data_AC.xlsx
+++ b/Historical_data_AC.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6450e5a01e7561fa/Desktop/ONG_proyectopersonal/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{F7B9CE97-AC28-4472-9E04-A2F306659678}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{98D57DAD-A366-43BE-B74E-2A6B22B12204}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{34D6BA04-1AFF-4A7C-9B19-3A12058CBEFE}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{34D6BA04-1AFF-4A7C-9B19-3A12058CBEFE}"/>
   </bookViews>
   <sheets>
     <sheet name="All containers" sheetId="1" r:id="rId1"/>
     <sheet name="Material" sheetId="2" r:id="rId2"/>
+    <sheet name="Countries coordinates" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="59">
   <si>
     <t>Numero Contenedor</t>
   </si>
@@ -205,6 +206,18 @@
   </si>
   <si>
     <t>Material enviado</t>
+  </si>
+  <si>
+    <t>Country</t>
+  </si>
+  <si>
+    <t>Latitude</t>
+  </si>
+  <si>
+    <t>Longitude</t>
+  </si>
+  <si>
+    <t>Perú</t>
   </si>
 </sst>
 </file>
@@ -5928,4 +5941,487 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE55D653-3B6D-48C5-A45F-119C8615AE3D}">
+  <dimension ref="A1:C43"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2">
+        <v>-8.8390000000000004</v>
+      </c>
+      <c r="C2">
+        <v>13.289400000000001</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3">
+        <v>28.033899999999999</v>
+      </c>
+      <c r="C3">
+        <v>1.6596</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>9.3077000000000005</v>
+      </c>
+      <c r="C4">
+        <v>2.3157999999999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5">
+        <v>12.238300000000001</v>
+      </c>
+      <c r="C5">
+        <v>-1.5616000000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6">
+        <v>-3.3731</v>
+      </c>
+      <c r="C6">
+        <v>29.918900000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7">
+        <v>16.538799999999998</v>
+      </c>
+      <c r="C7">
+        <v>-23.041799999999999</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8">
+        <v>7.3696999999999999</v>
+      </c>
+      <c r="C8">
+        <v>12.354699999999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9">
+        <v>-0.22800000000000001</v>
+      </c>
+      <c r="C9">
+        <v>15.8277</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10">
+        <v>21.521799999999999</v>
+      </c>
+      <c r="C10">
+        <v>-77.781199999999998</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B11">
+        <v>40.463700000000003</v>
+      </c>
+      <c r="C11">
+        <v>-3.7492000000000001</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>40</v>
+      </c>
+      <c r="B12">
+        <v>9.1449999999999996</v>
+      </c>
+      <c r="C12">
+        <v>40.489699999999999</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>39</v>
+      </c>
+      <c r="B13">
+        <v>13.443199999999999</v>
+      </c>
+      <c r="C13">
+        <v>-15.3101</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>25</v>
+      </c>
+      <c r="B14">
+        <v>7.9465000000000003</v>
+      </c>
+      <c r="C14">
+        <v>-1.0232000000000001</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>27</v>
+      </c>
+      <c r="B15">
+        <v>39.074199999999998</v>
+      </c>
+      <c r="C15">
+        <v>21.824300000000001</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16">
+        <v>15.7835</v>
+      </c>
+      <c r="C16">
+        <v>-90.230800000000002</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>29</v>
+      </c>
+      <c r="B17">
+        <v>9.9456000000000007</v>
+      </c>
+      <c r="C17">
+        <v>-9.6966000000000001</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>34</v>
+      </c>
+      <c r="B18">
+        <v>11.803699999999999</v>
+      </c>
+      <c r="C18">
+        <v>-15.180400000000001</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>35</v>
+      </c>
+      <c r="B19">
+        <v>1.6508</v>
+      </c>
+      <c r="C19">
+        <v>10.267899999999999</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>13</v>
+      </c>
+      <c r="B20">
+        <v>15.2</v>
+      </c>
+      <c r="C20">
+        <v>-86.241900000000001</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>14</v>
+      </c>
+      <c r="B21">
+        <v>20.593699999999998</v>
+      </c>
+      <c r="C21">
+        <v>78.962900000000005</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>4</v>
+      </c>
+      <c r="B22">
+        <v>-2.3599999999999999E-2</v>
+      </c>
+      <c r="C22">
+        <v>37.906199999999998</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>30</v>
+      </c>
+      <c r="B23">
+        <v>33.854700000000001</v>
+      </c>
+      <c r="C23">
+        <v>35.862299999999998</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>26</v>
+      </c>
+      <c r="B24">
+        <v>6.4280999999999997</v>
+      </c>
+      <c r="C24">
+        <v>-9.4295000000000009</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>41</v>
+      </c>
+      <c r="B25">
+        <v>-18.7669</v>
+      </c>
+      <c r="C25">
+        <v>46.869100000000003</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>36</v>
+      </c>
+      <c r="B26">
+        <v>-13.254300000000001</v>
+      </c>
+      <c r="C26">
+        <v>34.301499999999997</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>28</v>
+      </c>
+      <c r="B27">
+        <v>17.570699999999999</v>
+      </c>
+      <c r="C27">
+        <v>-3.9962</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>19</v>
+      </c>
+      <c r="B28">
+        <v>-18.665700000000001</v>
+      </c>
+      <c r="C28">
+        <v>35.529600000000002</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>42</v>
+      </c>
+      <c r="B29">
+        <v>31.952200000000001</v>
+      </c>
+      <c r="C29">
+        <v>35.233199999999997</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>58</v>
+      </c>
+      <c r="B30">
+        <v>-9.19</v>
+      </c>
+      <c r="C30">
+        <v>-75.015199999999993</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>32</v>
+      </c>
+      <c r="B31">
+        <v>6.6111000000000004</v>
+      </c>
+      <c r="C31">
+        <v>20.939399999999999</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>20</v>
+      </c>
+      <c r="B32">
+        <v>-4.0382999999999996</v>
+      </c>
+      <c r="C32">
+        <v>21.758700000000001</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>9</v>
+      </c>
+      <c r="B33">
+        <v>18.735700000000001</v>
+      </c>
+      <c r="C33">
+        <v>-70.162700000000001</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>10</v>
+      </c>
+      <c r="B34">
+        <v>14.497400000000001</v>
+      </c>
+      <c r="C34">
+        <v>-14.452400000000001</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>12</v>
+      </c>
+      <c r="B35">
+        <v>8.4605999999999995</v>
+      </c>
+      <c r="C35">
+        <v>-11.7799</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>24</v>
+      </c>
+      <c r="B36">
+        <v>34.802100000000003</v>
+      </c>
+      <c r="C36">
+        <v>38.9968</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>17</v>
+      </c>
+      <c r="B37">
+        <v>-6.3689999999999998</v>
+      </c>
+      <c r="C37">
+        <v>34.888800000000003</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>6</v>
+      </c>
+      <c r="B38">
+        <v>8.6195000000000004</v>
+      </c>
+      <c r="C38">
+        <v>0.82479999999999998</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>33</v>
+      </c>
+      <c r="B39">
+        <v>48.379399999999997</v>
+      </c>
+      <c r="C39">
+        <v>31.165600000000001</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>43</v>
+      </c>
+      <c r="B40">
+        <v>1.3733</v>
+      </c>
+      <c r="C40">
+        <v>32.290300000000002</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>11</v>
+      </c>
+      <c r="B41">
+        <v>-32.522799999999997</v>
+      </c>
+      <c r="C41">
+        <v>-55.765799999999999</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>7</v>
+      </c>
+      <c r="B42">
+        <v>6.4238</v>
+      </c>
+      <c r="C42">
+        <v>-66.589699999999993</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>44</v>
+      </c>
+      <c r="B43">
+        <v>14.058299999999999</v>
+      </c>
+      <c r="C43">
+        <v>108.27719999999999</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>